<commit_message>
Made skill to value calculation updates
</commit_message>
<xml_diff>
--- a/Resources/SkillToValue.xlsx
+++ b/Resources/SkillToValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aaron\Documents\Unity\Projects\unity-kings-of-the-beach\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0164DC32-427D-4904-A6FE-4A66641F61DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C58BD2E-731B-4769-9CF1-C56BF6228605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4706" yWindow="5391" windowWidth="19200" windowHeight="10072" xr2:uid="{ADB89B2A-C081-4CFC-9508-3215388A7CC4}"/>
+    <workbookView xWindow="9291" yWindow="4594" windowWidth="21823" windowHeight="13012" xr2:uid="{ADB89B2A-C081-4CFC-9508-3215388A7CC4}"/>
   </bookViews>
   <sheets>
     <sheet name="SkillToValue" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Skill</t>
   </si>
@@ -54,6 +54,21 @@
   </si>
   <si>
     <t>Skill to Value</t>
+  </si>
+  <si>
+    <t>Lerp</t>
+  </si>
+  <si>
+    <t>Lerp(t)</t>
+  </si>
+  <si>
+    <t>Full</t>
+  </si>
+  <si>
+    <t>Validated!</t>
+  </si>
+  <si>
+    <t>Can't use Lerp because it's sorta twice</t>
   </si>
 </sst>
 </file>
@@ -61,7 +76,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -94,7 +109,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,7 +444,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{353AE45F-2459-4C1F-BACE-432CF1F1F29A}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10.765625" bestFit="1" customWidth="1"/>
@@ -459,10 +474,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
@@ -479,7 +494,44 @@
       </c>
       <c r="B6" s="1">
         <f>(B4-B2)*(C3-B3)/(C2-B2)+B3</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <f>(B4-B2)/(C2-B2)</f>
         <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10">
+        <f>B3+(C3-B3)*B9</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11">
+        <f>B3+(C3-B3)*(B4-B2)/(C2-B2)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>